<commit_message>
Updated PROD Reports and RBU reports
</commit_message>
<xml_diff>
--- a/data/internalStats2/RebateRefreshOutput/Consolidated_Report_27JulPROD.xlsx
+++ b/data/internalStats2/RebateRefreshOutput/Consolidated_Report_27JulPROD.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TC4" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,12 +27,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCCC"/>
+        <bgColor rgb="00FFCCCC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +53,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,6 +430,320 @@
           <t>Table</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>specialty - brand only</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>specialty - rebatable</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>overall - brand only</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>non-specialty - brand only</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mail non-specialty - non rebatable (brand only)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>retail 30 non-specialty - non rebatable (brand only)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>overall - non rebatable (brand only)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>excl - generic</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>retail 90 non-specialty - rebatable</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>specialty - non rebatable (brand only)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>exclusions</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>start date:</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>overall - non rebatable (brand only)_22</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>retail 30 non-specialty - rebatable</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>w exclusions</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>retail 90 non-specialty - non rebatable (brand only)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>overall - rebatable</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>conservatism</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>excl - total</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mail non-specialty - rebatable</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>start date:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Start Date:</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>01/01/2025</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Start Date:</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>45658</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>End Date:</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>11/30/2025</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>End Date:</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>45991</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Total Months:</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Total Months:</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>